<commit_message>
validate follow_up_note and update formatting guidance release date
</commit_message>
<xml_diff>
--- a/test/fixtures/files/Sara-Alert-Format-Invalid-Fields.xlsx
+++ b/test/fixtures/files/Sara-Alert-Format-Invalid-Fields.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/twong/Documents/SARA-ALERT/SaraAlert/test/fixtures/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D14D5792-C6AE-5B46-AEF4-B3679A1406FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AF5F0C4-F69B-444E-B462-29C1158648B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="460" windowWidth="33600" windowHeight="19380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="258">
   <si>
     <t>First Name</t>
   </si>
@@ -791,6 +791,9 @@
   </si>
   <si>
     <t>invalid reason</t>
+  </si>
+  <si>
+    <t>note</t>
   </si>
 </sst>
 </file>
@@ -1886,6 +1889,9 @@
       <c r="DH3" t="s">
         <v>252</v>
       </c>
+      <c r="DJ3" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="4" spans="1:114" x14ac:dyDescent="0.15">
       <c r="A4" t="s">

</xml_diff>